<commit_message>
Corte de chapa: tipo de cambio fijo 1420, 20 golpes por minuto confirmados y sin pendientes de planos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/Comparacion_corte.xlsx
+++ b/salida/Comparacion_corte.xlsx
@@ -217,7 +217,7 @@
     <t xml:space="preserve">ARS/USD</t>
   </si>
   <si>
-    <t xml:space="preserve">Pradecon, presupuestos 173170 y 173195 (28/09/2026).</t>
+    <t xml:space="preserve">Valor fijo del proyecto (criterio del grupo).</t>
   </si>
   <si>
     <t xml:space="preserve">Costo hora de operario</t>
@@ -319,7 +319,7 @@
     <t xml:space="preserve">Guillotina 2 (piezas) QC12Y 6 × 2500: golpes por minuto</t>
   </si>
   <si>
-    <t xml:space="preserve">La publicación del link no lo da: dato de la HG 6 × 2500 en la ficha Molinari Panther. Confirmar.</t>
+    <t xml:space="preserve">Confirmado por el grupo (igual que la HG 6 × 2500 de la ficha Molinari Panther).</t>
   </si>
   <si>
     <t xml:space="preserve">Guillotina 2: largo de corte para franjas en paralelo</t>
@@ -997,7 +997,7 @@
     <t xml:space="preserve">Plano extintor rodante 100 kg R1 (Ø390)</t>
   </si>
   <si>
-    <t xml:space="preserve">Alto: cuerpo del modelo 3D del plano (incluye el labio del encastre). 1 kg en chapa de 0,9 mm por decisión del grupo; el plano G809 todavía lo da en caño de 1,25 mm.</t>
+    <t xml:space="preserve">Alto: cuerpo del modelo 3D del plano (incluye el labio del encastre). 1 kg en chapa de 0,9 mm por decisión del grupo.</t>
   </si>
   <si>
     <t xml:space="preserve">B) Discos: igual superficie que la pieza embutida (sin sobremedida de recorte)</t>
@@ -2199,19 +2199,19 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>1151075.98042224</c:v>
+                  <c:v>1151596.9920884</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1149876.75672962</c:v>
+                  <c:v>1150161.11678637</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1202673.06421411</c:v>
+                  <c:v>1203055.32553162</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1120950.50711101</c:v>
+                  <c:v>1121061.70588396</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1029258.77124521</c:v>
+                  <c:v>1029277.71500999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2219,11 +2219,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="31146617"/>
-        <c:axId val="36843715"/>
+        <c:axId val="59415577"/>
+        <c:axId val="84153763"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="31146617"/>
+        <c:axId val="59415577"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2255,7 +2255,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36843715"/>
+        <c:crossAx val="84153763"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2263,7 +2263,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="36843715"/>
+        <c:axId val="84153763"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -2340,7 +2340,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="31146617"/>
+        <c:crossAx val="59415577"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2768,23 +2768,23 @@
       </c>
       <c r="B11" s="5" t="n">
         <f aca="false">INDEX(Cálculo!$C$44:$L$44,Datos!$B$6-2025)</f>
-        <v>512456.973400222</v>
+        <v>512740.555165235</v>
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">INDEX(Cálculo!$C$67:$L$67,Datos!$B$6-2025)</f>
-        <v>566015.874480069</v>
+        <v>566169.097545704</v>
       </c>
       <c r="D11" s="5" t="n">
         <f aca="false">INDEX(Cálculo!$C$93:$L$93,Datos!$B$6-2025)</f>
-        <v>523407.396571221</v>
+        <v>523613.790553217</v>
       </c>
       <c r="E11" s="5" t="n">
         <f aca="false">INDEX(Cálculo!$C$105:$L$105,Datos!$B$6-2025)</f>
-        <v>542213.909148228</v>
+        <v>542274.009727035</v>
       </c>
       <c r="F11" s="5" t="n">
         <f aca="false">INDEX(Cálculo!$C$119:$L$119,Datos!$B$6-2025)</f>
-        <v>539381.740510096</v>
+        <v>539391.983464073</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2793,23 +2793,23 @@
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">B7+SUMPRODUCT(Cálculo!$C$44:$L$44,Cálculo!$C$6:$L$6)</f>
-        <v>1151075.98042224</v>
+        <v>1151596.9920884</v>
       </c>
       <c r="C12" s="8" t="n">
         <f aca="false">C7+SUMPRODUCT(Cálculo!$C$67:$L$67,Cálculo!$C$6:$L$6)</f>
-        <v>1149876.75672962</v>
+        <v>1150161.11678637</v>
       </c>
       <c r="D12" s="8" t="n">
         <f aca="false">D7+SUMPRODUCT(Cálculo!$C$93:$L$93,Cálculo!$C$6:$L$6)</f>
-        <v>1202673.06421411</v>
+        <v>1203055.32553162</v>
       </c>
       <c r="E12" s="8" t="n">
         <f aca="false">E7+SUMPRODUCT(Cálculo!$C$105:$L$105,Cálculo!$C$6:$L$6)</f>
-        <v>1120950.50711101</v>
+        <v>1121061.70588396</v>
       </c>
       <c r="F12" s="8" t="n">
         <f aca="false">F7+SUMPRODUCT(Cálculo!$C$119:$L$119,Cálculo!$C$6:$L$6)</f>
-        <v>1029258.77124521</v>
+        <v>1029277.71500999</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2842,15 +2842,15 @@
       </c>
       <c r="B14" s="5" t="n">
         <f aca="false">B12-MIN($B$12:$E$12)</f>
-        <v>30125.4733112331</v>
+        <v>30535.2862044449</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">C12-MIN($B$12:$E$12)</f>
-        <v>28926.2496186085</v>
+        <v>29099.410902411</v>
       </c>
       <c r="D14" s="5" t="n">
         <f aca="false">D12-MIN($B$12:$E$12)</f>
-        <v>81722.5571030972</v>
+        <v>81993.6196476619</v>
       </c>
       <c r="E14" s="5" t="n">
         <f aca="false">E12-MIN($B$12:$E$12)</f>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="F14" s="5" t="n">
         <f aca="false">F12-MIN($B$12:$E$12)</f>
-        <v>-91691.7358658053</v>
+        <v>-91783.9908739689</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="B17" s="6" t="n">
         <f aca="false">($B$12-$E$12)/SUMPRODUCT(Cálculo!$C$52:$L$52,Cálculo!$C$6:$L$6)</f>
-        <v>0.0376223796501009</v>
+        <v>0.0381341769617858</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="B18" s="6" t="n">
         <f aca="false">($C$12-$E$12)/SUMPRODUCT(Cálculo!$C$31:$L$31,Cálculo!$C$6:$L$6)</f>
-        <v>0.128181797519102</v>
+        <v>0.128949132549089</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3119,7 +3119,7 @@
         <v>61</v>
       </c>
       <c r="B14" s="16" t="n">
-        <v>1545</v>
+        <v>1420</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>62</v>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="B15" s="18" t="n">
         <f aca="false">Datos!$B$11/Datos!$B$12/Datos!$B$14</f>
-        <v>5.77312621359223</v>
+        <v>6.28132394366197</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>65</v>
@@ -13573,43 +13573,43 @@
       </c>
       <c r="C42" s="5" t="n">
         <f aca="false">C41*Datos!$B$15</f>
-        <v>79.2411617388321</v>
+        <v>86.2166161172504</v>
       </c>
       <c r="D42" s="5" t="n">
         <f aca="false">D41*Datos!$B$15</f>
-        <v>126.299757493973</v>
+        <v>137.417693893091</v>
       </c>
       <c r="E42" s="5" t="n">
         <f aca="false">E41*Datos!$B$15</f>
-        <v>263.047892657325</v>
+        <v>286.203517010962</v>
       </c>
       <c r="F42" s="5" t="n">
         <f aca="false">F41*Datos!$B$15</f>
-        <v>575.686105744984</v>
+        <v>626.362699560564</v>
       </c>
       <c r="G42" s="5" t="n">
         <f aca="false">G41*Datos!$B$15</f>
-        <v>1000.46841110002</v>
+        <v>1088.53781348558</v>
       </c>
       <c r="H42" s="5" t="n">
         <f aca="false">H41*Datos!$B$15</f>
-        <v>1404.6406358258</v>
+        <v>1528.28857912032</v>
       </c>
       <c r="I42" s="5" t="n">
         <f aca="false">I41*Datos!$B$15</f>
-        <v>1934.05844588634</v>
+        <v>2104.31006964394</v>
       </c>
       <c r="J42" s="5" t="n">
         <f aca="false">J41*Datos!$B$15</f>
-        <v>2469.43529358963</v>
+        <v>2686.81516098309</v>
       </c>
       <c r="K42" s="5" t="n">
         <f aca="false">K41*Datos!$B$15</f>
-        <v>2787.97313013097</v>
+        <v>3033.39330003687</v>
       </c>
       <c r="L42" s="5" t="n">
         <f aca="false">L41*Datos!$B$15</f>
-        <v>3221.48885055494</v>
+        <v>3505.07061556858</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13669,43 +13669,43 @@
       </c>
       <c r="C44" s="8" t="n">
         <f aca="false">C33+C35+C39+C42+C43</f>
-        <v>21075.2804988648</v>
+        <v>21082.2559532432</v>
       </c>
       <c r="D44" s="8" t="n">
         <f aca="false">D33+D35+D39+D42+D43</f>
-        <v>31902.6766684887</v>
+        <v>31913.7946048878</v>
       </c>
       <c r="E44" s="8" t="n">
         <f aca="false">E33+E35+E39+E42+E43</f>
-        <v>53832.7049640657</v>
+        <v>53855.8605884193</v>
       </c>
       <c r="F44" s="8" t="n">
         <f aca="false">F33+F35+F39+F42+F43</f>
-        <v>100177.666761432</v>
+        <v>100228.343355248</v>
       </c>
       <c r="G44" s="8" t="n">
         <f aca="false">G33+G35+G39+G42+G43</f>
-        <v>167174.731409601</v>
+        <v>167262.800811987</v>
       </c>
       <c r="H44" s="8" t="n">
         <f aca="false">H33+H35+H39+H42+H43</f>
-        <v>231324.442882778</v>
+        <v>231448.090826072</v>
       </c>
       <c r="I44" s="8" t="n">
         <f aca="false">I33+I35+I39+I42+I43</f>
-        <v>311332.485199816</v>
+        <v>311502.736823574</v>
       </c>
       <c r="J44" s="8" t="n">
         <f aca="false">J33+J35+J39+J42+J43</f>
-        <v>392972.73664664</v>
+        <v>393190.116514033</v>
       </c>
       <c r="K44" s="8" t="n">
         <f aca="false">K33+K35+K39+K42+K43</f>
-        <v>444927.302442415</v>
+        <v>445172.722612321</v>
       </c>
       <c r="L44" s="8" t="n">
         <f aca="false">L33+L35+L39+L42+L43</f>
-        <v>512456.973400222</v>
+        <v>512740.555165235</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14586,43 +14586,43 @@
       </c>
       <c r="C65" s="5" t="n">
         <f aca="false">C64*Datos!$B$15</f>
-        <v>47.9542384133862</v>
+        <v>52.1755622173815</v>
       </c>
       <c r="D65" s="5" t="n">
         <f aca="false">D64*Datos!$B$15</f>
-        <v>78.9641870104958</v>
+        <v>85.9152598107155</v>
       </c>
       <c r="E65" s="5" t="n">
         <f aca="false">E64*Datos!$B$15</f>
-        <v>153.440849070587</v>
+        <v>166.947966066237</v>
       </c>
       <c r="F65" s="5" t="n">
         <f aca="false">F64*Datos!$B$15</f>
-        <v>317.112614654582</v>
+        <v>345.027457493893</v>
       </c>
       <c r="G65" s="5" t="n">
         <f aca="false">G64*Datos!$B$15</f>
-        <v>546.173694910134</v>
+        <v>594.25236523673</v>
       </c>
       <c r="H65" s="5" t="n">
         <f aca="false">H64*Datos!$B$15</f>
-        <v>765.495869473907</v>
+        <v>832.88106925154</v>
       </c>
       <c r="I65" s="5" t="n">
         <f aca="false">I64*Datos!$B$15</f>
-        <v>1047.09092288656</v>
+        <v>1139.26441961953</v>
       </c>
       <c r="J65" s="5" t="n">
         <f aca="false">J64*Datos!$B$15</f>
-        <v>1332.82258858243</v>
+        <v>1450.14852067596</v>
       </c>
       <c r="K65" s="5" t="n">
         <f aca="false">K64*Datos!$B$15</f>
-        <v>1507.7035023122</v>
+        <v>1640.42388103687</v>
       </c>
       <c r="L65" s="5" t="n">
         <f aca="false">L64*Datos!$B$15</f>
-        <v>1740.61402560734</v>
+        <v>1893.83709124179</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14682,43 +14682,43 @@
       </c>
       <c r="C67" s="8" t="n">
         <f aca="false">C59+C61+C63+C65+C66</f>
-        <v>20087.5188687993</v>
+        <v>20091.7401926033</v>
       </c>
       <c r="D67" s="8" t="n">
         <f aca="false">D59+D61+D63+D65+D66</f>
-        <v>32027.1475264932</v>
+        <v>32034.0985992934</v>
       </c>
       <c r="E67" s="8" t="n">
         <f aca="false">E59+E61+E63+E65+E66</f>
-        <v>56156.8736250397</v>
+        <v>56170.3807420354</v>
       </c>
       <c r="F67" s="8" t="n">
         <f aca="false">F59+F61+F63+F65+F66</f>
-        <v>107091.045366794</v>
+        <v>107118.960209633</v>
       </c>
       <c r="G67" s="8" t="n">
         <f aca="false">G59+G61+G63+G65+G66</f>
-        <v>180879.361226597</v>
+        <v>180927.439896924</v>
       </c>
       <c r="H67" s="8" t="n">
         <f aca="false">H59+H61+H63+H65+H66</f>
-        <v>252282.661309645</v>
+        <v>252350.046509423</v>
       </c>
       <c r="I67" s="8" t="n">
         <f aca="false">I59+I61+I63+I65+I66</f>
-        <v>341562.400485841</v>
+        <v>341654.573982574</v>
       </c>
       <c r="J67" s="8" t="n">
         <f aca="false">J59+J61+J63+J65+J66</f>
-        <v>432660.526100038</v>
+        <v>432777.852032131</v>
       </c>
       <c r="K67" s="8" t="n">
         <f aca="false">K59+K61+K63+K65+K66</f>
-        <v>490663.413322053</v>
+        <v>490796.133700777</v>
       </c>
       <c r="L67" s="8" t="n">
         <f aca="false">L59+L61+L63+L65+L66</f>
-        <v>566015.874480069</v>
+        <v>566169.097545704</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15743,43 +15743,43 @@
       </c>
       <c r="C91" s="5" t="n">
         <f aca="false">C90*Datos!$B$15</f>
-        <v>63.5399583657207</v>
+        <v>69.1332645598863</v>
       </c>
       <c r="D91" s="5" t="n">
         <f aca="false">D90*Datos!$B$15</f>
-        <v>105.890089837629</v>
+        <v>115.211400562773</v>
       </c>
       <c r="E91" s="5" t="n">
         <f aca="false">E90*Datos!$B$15</f>
-        <v>205.382698417886</v>
+        <v>223.462161306784</v>
       </c>
       <c r="F91" s="5" t="n">
         <f aca="false">F90*Datos!$B$15</f>
-        <v>425.690510644883</v>
+        <v>463.163266863623</v>
       </c>
       <c r="G91" s="5" t="n">
         <f aca="false">G90*Datos!$B$15</f>
-        <v>731.841291228295</v>
+        <v>796.263940104025</v>
       </c>
       <c r="H91" s="5" t="n">
         <f aca="false">H90*Datos!$B$15</f>
-        <v>1027.90818678814</v>
+        <v>1118.39306238569</v>
       </c>
       <c r="I91" s="5" t="n">
         <f aca="false">I90*Datos!$B$15</f>
-        <v>1408.40765117416</v>
+        <v>1532.38719793245</v>
       </c>
       <c r="J91" s="5" t="n">
         <f aca="false">J90*Datos!$B$15</f>
-        <v>1795.01163512555</v>
+        <v>1953.02322272463</v>
       </c>
       <c r="K91" s="5" t="n">
         <f aca="false">K90*Datos!$B$15</f>
-        <v>2028.80209234706</v>
+        <v>2207.39382582831</v>
       </c>
       <c r="L91" s="5" t="n">
         <f aca="false">L90*Datos!$B$15</f>
-        <v>2344.63563546944</v>
+        <v>2551.02961746499</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15839,43 +15839,43 @@
       </c>
       <c r="C93" s="8" t="n">
         <f aca="false">C83+C85+C87+C91+C92</f>
-        <v>22376.4728460117</v>
+        <v>22382.0661522059</v>
       </c>
       <c r="D93" s="8" t="n">
         <f aca="false">D83+D85+D87+D91+D92</f>
-        <v>33977.1719364068</v>
+        <v>33986.4932471319</v>
       </c>
       <c r="E93" s="8" t="n">
         <f aca="false">E83+E85+E87+E91+E92</f>
-        <v>56596.3525871409</v>
+        <v>56614.4320500298</v>
       </c>
       <c r="F93" s="8" t="n">
         <f aca="false">F83+F85+F87+F91+F92</f>
-        <v>104152.033182019</v>
+        <v>104189.505938238</v>
       </c>
       <c r="G93" s="8" t="n">
         <f aca="false">G83+G85+G87+G91+G92</f>
-        <v>172524.689982872</v>
+        <v>172589.112631748</v>
       </c>
       <c r="H93" s="8" t="n">
         <f aca="false">H83+H85+H87+H91+H92</f>
-        <v>237881.704764455</v>
+        <v>237972.189640053</v>
       </c>
       <c r="I93" s="8" t="n">
         <f aca="false">I83+I85+I87+I91+I92</f>
-        <v>319454.29813043</v>
+        <v>319578.277677188</v>
       </c>
       <c r="J93" s="8" t="n">
         <f aca="false">J83+J85+J87+J91+J92</f>
-        <v>402708.39137186</v>
+        <v>402866.402959459</v>
       </c>
       <c r="K93" s="8" t="n">
         <f aca="false">K83+K85+K87+K91+K92</f>
-        <v>454907.91465514</v>
+        <v>455086.506388621</v>
       </c>
       <c r="L93" s="8" t="n">
         <f aca="false">L83+L85+L87+L91+L92</f>
-        <v>523407.396571221</v>
+        <v>523613.790553217</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16228,43 +16228,43 @@
       </c>
       <c r="C103" s="5" t="n">
         <f aca="false">C102*Datos!$B$15</f>
-        <v>18.2193017724389</v>
+        <v>19.8231135481817</v>
       </c>
       <c r="D103" s="5" t="n">
         <f aca="false">D102*Datos!$B$15</f>
-        <v>29.980987410963</v>
+        <v>32.6201588379844</v>
       </c>
       <c r="E103" s="5" t="n">
         <f aca="false">E102*Datos!$B$15</f>
-        <v>59.1103731094459</v>
+        <v>64.3137510240098</v>
       </c>
       <c r="F103" s="5" t="n">
         <f aca="false">F102*Datos!$B$15</f>
-        <v>123.718856895404</v>
+        <v>134.609601340422</v>
       </c>
       <c r="G103" s="5" t="n">
         <f aca="false">G102*Datos!$B$15</f>
-        <v>213.466121210214</v>
+        <v>232.257153006888</v>
       </c>
       <c r="H103" s="5" t="n">
         <f aca="false">H102*Datos!$B$15</f>
-        <v>299.562157651164</v>
+        <v>325.932065895105</v>
       </c>
       <c r="I103" s="5" t="n">
         <f aca="false">I102*Datos!$B$15</f>
-        <v>410.137921044242</v>
+        <v>446.241611277009</v>
       </c>
       <c r="J103" s="5" t="n">
         <f aca="false">J102*Datos!$B$15</f>
-        <v>522.391040910551</v>
+        <v>568.376167751268</v>
       </c>
       <c r="K103" s="5" t="n">
         <f aca="false">K102*Datos!$B$15</f>
-        <v>591.003247985711</v>
+        <v>643.02818178727</v>
       </c>
       <c r="L103" s="5" t="n">
         <f aca="false">L102*Datos!$B$15</f>
-        <v>682.742575239051</v>
+        <v>742.843154045305</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16324,43 +16324,43 @@
       </c>
       <c r="C105" s="8" t="n">
         <f aca="false">C97+C99+C101+C103+C104</f>
-        <v>19761.4915882695</v>
+        <v>19763.0954000452</v>
       </c>
       <c r="D105" s="8" t="n">
         <f aca="false">D97+D99+D101+D103+D104</f>
-        <v>31174.6160904509</v>
+        <v>31177.2552618779</v>
       </c>
       <c r="E105" s="8" t="n">
         <f aca="false">E97+E99+E101+E103+E104</f>
-        <v>54310.1678946896</v>
+        <v>54315.3712726041</v>
       </c>
       <c r="F105" s="8" t="n">
         <f aca="false">F97+F99+F101+F103+F104</f>
-        <v>103196.666741091</v>
+        <v>103207.557485536</v>
       </c>
       <c r="G105" s="8" t="n">
         <f aca="false">G97+G99+G101+G103+G104</f>
-        <v>173927.968717565</v>
+        <v>173946.759749362</v>
       </c>
       <c r="H105" s="8" t="n">
         <f aca="false">H97+H99+H101+H103+H104</f>
-        <v>242207.854064306</v>
+        <v>242234.22397255</v>
       </c>
       <c r="I105" s="8" t="n">
         <f aca="false">I97+I99+I101+I103+I104</f>
-        <v>327601.335441653</v>
+        <v>327637.439131886</v>
       </c>
       <c r="J105" s="8" t="n">
         <f aca="false">J97+J99+J101+J103+J104</f>
-        <v>414719.857955511</v>
+        <v>414765.843082351</v>
       </c>
       <c r="K105" s="8" t="n">
         <f aca="false">K97+K99+K101+K103+K104</f>
-        <v>470162.876687393</v>
+        <v>470214.901621195</v>
       </c>
       <c r="L105" s="8" t="n">
         <f aca="false">L97+L99+L101+L103+L104</f>
-        <v>542213.909148228</v>
+        <v>542274.009727035</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16809,43 +16809,43 @@
       </c>
       <c r="C117" s="5" t="n">
         <f aca="false">C116*Datos!$B$15</f>
-        <v>3.03120711424153</v>
+        <v>3.29803872641068</v>
       </c>
       <c r="D117" s="5" t="n">
         <f aca="false">D116*Datos!$B$15</f>
-        <v>5.30854563147023</v>
+        <v>5.77584718353627</v>
       </c>
       <c r="E117" s="5" t="n">
         <f aca="false">E116*Datos!$B$15</f>
-        <v>10.2915784768417</v>
+        <v>11.1975272864228</v>
       </c>
       <c r="F117" s="5" t="n">
         <f aca="false">F116*Datos!$B$15</f>
-        <v>21.1314859309091</v>
+        <v>22.991651945954</v>
       </c>
       <c r="G117" s="5" t="n">
         <f aca="false">G116*Datos!$B$15</f>
-        <v>36.3058538646068</v>
+        <v>39.501791704801</v>
       </c>
       <c r="H117" s="5" t="n">
         <f aca="false">H116*Datos!$B$15</f>
-        <v>51.166163194614</v>
+        <v>55.6702268561117</v>
       </c>
       <c r="I117" s="5" t="n">
         <f aca="false">I116*Datos!$B$15</f>
-        <v>69.6424128335696</v>
+        <v>75.7729069210317</v>
       </c>
       <c r="J117" s="5" t="n">
         <f aca="false">J116*Datos!$B$15</f>
-        <v>88.543264239013</v>
+        <v>96.3375656685035</v>
       </c>
       <c r="K117" s="5" t="n">
         <f aca="false">K116*Datos!$B$15</f>
-        <v>100.541020712267</v>
+        <v>109.391462676375</v>
       </c>
       <c r="L117" s="5" t="n">
         <f aca="false">L116*Datos!$B$15</f>
-        <v>116.359957172203</v>
+        <v>126.60291114863</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16905,43 +16905,43 @@
       </c>
       <c r="C119" s="8" t="n">
         <f aca="false">C111+C113+C115+C117+C118</f>
-        <v>17445.1218393196</v>
+        <v>17445.3886709318</v>
       </c>
       <c r="D119" s="8" t="n">
         <f aca="false">D111+D113+D115+D117+D118</f>
-        <v>28960.7119952788</v>
+        <v>28961.1792968309</v>
       </c>
       <c r="E119" s="8" t="n">
         <f aca="false">E111+E113+E115+E117+E118</f>
-        <v>52095.3488432993</v>
+        <v>52096.2547921089</v>
       </c>
       <c r="F119" s="8" t="n">
         <f aca="false">F111+F113+F115+F117+F118</f>
-        <v>100863.573816992</v>
+        <v>100865.433983007</v>
       </c>
       <c r="G119" s="8" t="n">
         <f aca="false">G111+G113+G115+G117+G118</f>
-        <v>171519.399542673</v>
+        <v>171522.595480513</v>
       </c>
       <c r="H119" s="8" t="n">
         <f aca="false">H111+H113+H115+H117+H118</f>
-        <v>239770.383009653</v>
+        <v>239774.887073314</v>
       </c>
       <c r="I119" s="8" t="n">
         <f aca="false">I111+I113+I115+I117+I118</f>
-        <v>324990.497299015</v>
+        <v>324996.627793102</v>
       </c>
       <c r="J119" s="8" t="n">
         <f aca="false">J111+J113+J115+J117+J118</f>
-        <v>411965.754970766</v>
+        <v>411973.549272195</v>
       </c>
       <c r="K119" s="8" t="n">
         <f aca="false">K111+K113+K115+K117+K118</f>
-        <v>467410.218893336</v>
+        <v>467419.0693353</v>
       </c>
       <c r="L119" s="8" t="n">
         <f aca="false">L111+L113+L115+L117+L118</f>
-        <v>539381.740510096</v>
+        <v>539391.983464073</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>